<commit_message>
happy cases run | expansion + negative cases pending
</commit_message>
<xml_diff>
--- a/sample_bills/output/medicine_bills.xlsx
+++ b/sample_bills/output/medicine_bills.xlsx
@@ -461,12 +461,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>14.09.2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lifecare Medicos</t>
+          <t>Lifecare</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -477,7 +477,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>